<commit_message>
Sprint 5: HU-117 servicios contratados y HU-125 imprimir OT (BD/430-431)
HU-117: alta, edición, baja e informe del proveedor en Orden_Trabajo_Servicio,
costo de terceros separado por moneda y cierre bloqueado sin informe. Se
registra desde la ficha de la OT, en un cajón.
HU-125: OrdenTrabajoImprimir.aspx (hoja A4 con encabezado del cliente, pasos,
repuestos, mano de obra, servicios, cierre y firmas) y botón Imprimir.
Sprint Backlog S5, Product Backlog y Pendientes sincronizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Product_Backlog_por_Sprint.xlsx
+++ b/Fase 2/SIGMA_Product_Backlog_por_Sprint.xlsx
@@ -58599,6 +58599,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="26">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -59093,7 +59094,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
@@ -59519,7 +59520,7 @@
       </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="N17" s="13" t="inlineStr">

</xml_diff>